<commit_message>
Added sample dates.py file
Code will later be used to get cohort dates for their respective workshop days
</commit_message>
<xml_diff>
--- a/class documents/roster.xlsx
+++ b/class documents/roster.xlsx
@@ -6,7 +6,7 @@
     <sheet state="visible" name="Class Roster" sheetId="1" r:id="rId4"/>
     <sheet state="visible" name="Student List" sheetId="2" r:id="rId5"/>
     <sheet state="visible" name="Demographic Data" sheetId="3" r:id="rId6"/>
-    <sheet state="visible" name="October 2025" sheetId="4" r:id="rId7"/>
+    <sheet state="visible" name="{Month} {Year}" sheetId="4" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="StudentName">#REF!</definedName>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="53">
   <si>
     <r>
       <rPr>
@@ -108,6 +108,25 @@
     <t xml:space="preserve">  </t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <rFont val="Bookman Old Style"/>
+        <b/>
+        <color rgb="FFFFFFFF"/>
+        <sz val="24.0"/>
+      </rPr>
+      <t>Dev/Mission HQ 360 Valencia - {Month} {Year}</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Century Gothic"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
+  <si>
     <t>STATUS</t>
   </si>
   <si>
@@ -126,10 +145,10 @@
     <t>Starting Date</t>
   </si>
   <si>
-    <t>Dia1</t>
+    <t>{Day1}</t>
   </si>
   <si>
-    <t>Dia2</t>
+    <t>{Day2}</t>
   </si>
   <si>
     <t>Present Days</t>
@@ -151,6 +170,30 @@
   </si>
   <si>
     <t xml:space="preserve">Last Name </t>
+  </si>
+  <si>
+    <t>{Date1}</t>
+  </si>
+  <si>
+    <t>{Date2}</t>
+  </si>
+  <si>
+    <t>{Date3}</t>
+  </si>
+  <si>
+    <t>{Date4}</t>
+  </si>
+  <si>
+    <t>{Date5}</t>
+  </si>
+  <si>
+    <t>{Date6}</t>
+  </si>
+  <si>
+    <t>{Date7}</t>
+  </si>
+  <si>
+    <t>{Date8}</t>
   </si>
   <si>
     <t>O</t>
@@ -175,11 +218,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="(###)###-####"/>
     <numFmt numFmtId="165" formatCode="(###) ###-####"/>
     <numFmt numFmtId="166" formatCode="M/d/yyyy"/>
-    <numFmt numFmtId="167" formatCode="m/d"/>
   </numFmts>
   <fonts count="17">
     <font>
@@ -537,7 +579,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="97">
+  <cellXfs count="96">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
@@ -790,9 +832,6 @@
     <xf borderId="12" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="12" fillId="0" fontId="12" numFmtId="167" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
     <xf borderId="24" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
@@ -842,88 +881,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>571500</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="10677525" cy="1457325"/>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="Shape 3"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="12000" y="3056100"/>
-          <a:ext cx="10668000" cy="1447800"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="3D85C6"/>
-        </a:solidFill>
-        <a:ln cap="flat" cmpd="sng" w="9525">
-          <a:solidFill>
-            <a:srgbClr val="3D85C6"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:round/>
-          <a:headEnd len="sm" w="sm" type="none"/>
-          <a:tailEnd len="sm" w="sm" type="none"/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr anchorCtr="0" anchor="ctr" bIns="91425" lIns="91425" spcFirstLastPara="1" rIns="91425" wrap="square" tIns="91425">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr indent="0" lvl="0" marL="0" rtl="0" algn="ctr">
-            <a:spcBef>
-              <a:spcPts val="0"/>
-            </a:spcBef>
-            <a:spcAft>
-              <a:spcPts val="0"/>
-            </a:spcAft>
-            <a:buClr>
-              <a:srgbClr val="FFFFFF"/>
-            </a:buClr>
-            <a:buSzPts val="3000"/>
-            <a:buFont typeface="Bookman Old Style"/>
-            <a:buNone/>
-          </a:pPr>
-          <a:r>
-            <a:rPr b="1" lang="en-US" sz="3000">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-              <a:latin typeface="Bookman Old Style"/>
-              <a:ea typeface="Bookman Old Style"/>
-              <a:cs typeface="Bookman Old Style"/>
-              <a:sym typeface="Bookman Old Style"/>
-            </a:rPr>
-            <a:t>Dev/Mission HQ 360 Valencia - October 2025</a:t>
-          </a:r>
-          <a:endParaRPr b="1" sz="3000">
-            <a:solidFill>
-              <a:srgbClr val="FFFFFF"/>
-            </a:solidFill>
-            <a:latin typeface="Bookman Old Style"/>
-            <a:ea typeface="Bookman Old Style"/>
-            <a:cs typeface="Bookman Old Style"/>
-            <a:sym typeface="Bookman Old Style"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -19381,19 +19339,29 @@
     <col customWidth="1" min="14" max="14" width="36.86"/>
   </cols>
   <sheetData>
-    <row r="2" ht="105.75" customHeight="1"/>
+    <row r="2" ht="105.75" customHeight="1">
+      <c r="D2" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="8"/>
+      <c r="J2" s="8"/>
+    </row>
     <row r="4">
       <c r="A4" s="49" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B4" s="49" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C4" s="49" t="s">
         <v>11</v>
       </c>
       <c r="D4" s="49" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E4" s="49" t="s">
         <v>14</v>
@@ -19408,10 +19376,10 @@
         <v>17</v>
       </c>
       <c r="I4" s="49" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="J4" s="49" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="K4" s="50" t="s">
         <v>19</v>
@@ -19664,6 +19632,9 @@
       <c r="M16" s="66"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="D2:J2"/>
+  </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
@@ -19682,7 +19653,7 @@
   <sheetData>
     <row r="3">
       <c r="B3" s="49" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C3" s="49" t="s">
         <v>11</v>
@@ -19697,10 +19668,10 @@
         <v>16</v>
       </c>
       <c r="G3" s="49" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H3" s="49" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I3" s="49" t="s">
         <v>18</v>
@@ -19869,7 +19840,7 @@
     </row>
     <row r="2">
       <c r="A2" s="72" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B2" s="73"/>
       <c r="C2" s="68"/>
@@ -19890,85 +19861,85 @@
       <c r="A3" s="75"/>
       <c r="B3" s="76"/>
       <c r="C3" s="77" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D3" s="77" t="s">
+        <v>31</v>
+      </c>
+      <c r="E3" s="77" t="s">
         <v>30</v>
       </c>
-      <c r="E3" s="77" t="s">
-        <v>29</v>
+      <c r="F3" s="77" t="s">
+        <v>31</v>
       </c>
-      <c r="F3" s="77" t="s">
+      <c r="G3" s="77" t="s">
         <v>30</v>
       </c>
-      <c r="G3" s="77" t="s">
-        <v>29</v>
+      <c r="H3" s="77" t="s">
+        <v>31</v>
       </c>
-      <c r="H3" s="77" t="s">
+      <c r="I3" s="77" t="s">
         <v>30</v>
       </c>
-      <c r="I3" s="77" t="s">
-        <v>29</v>
-      </c>
       <c r="J3" s="77" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="K3" s="78" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="L3" s="79" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="M3" s="80" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="N3" s="81" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="O3" s="82" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="83" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B4" s="83" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
-      <c r="C4" s="84">
-        <v>45950.0</v>
+      <c r="C4" s="77" t="s">
+        <v>39</v>
       </c>
-      <c r="D4" s="84">
-        <v>45952.0</v>
+      <c r="D4" s="77" t="s">
+        <v>40</v>
       </c>
-      <c r="E4" s="84">
-        <v>45957.0</v>
+      <c r="E4" s="77" t="s">
+        <v>41</v>
       </c>
-      <c r="F4" s="84">
-        <v>45959.0</v>
+      <c r="F4" s="77" t="s">
+        <v>42</v>
       </c>
-      <c r="G4" s="84">
-        <v>45964.0</v>
+      <c r="G4" s="77" t="s">
+        <v>43</v>
       </c>
-      <c r="H4" s="84">
-        <v>45966.0</v>
+      <c r="H4" s="77" t="s">
+        <v>44</v>
       </c>
-      <c r="I4" s="84">
-        <v>45971.0</v>
+      <c r="I4" s="77" t="s">
+        <v>45</v>
       </c>
-      <c r="J4" s="84">
-        <v>45973.0</v>
+      <c r="J4" s="77" t="s">
+        <v>46</v>
       </c>
-      <c r="K4" s="85"/>
-      <c r="L4" s="85"/>
-      <c r="M4" s="85"/>
-      <c r="N4" s="85"/>
-      <c r="O4" s="85"/>
+      <c r="K4" s="84"/>
+      <c r="L4" s="84"/>
+      <c r="M4" s="84"/>
+      <c r="N4" s="84"/>
+      <c r="O4" s="84"/>
     </row>
     <row r="5">
-      <c r="A5" s="86"/>
-      <c r="B5" s="87"/>
+      <c r="A5" s="85"/>
+      <c r="B5" s="86"/>
       <c r="C5" s="32"/>
       <c r="D5" s="32"/>
       <c r="E5" s="41"/>
@@ -19977,27 +19948,27 @@
       <c r="H5" s="41"/>
       <c r="I5" s="41"/>
       <c r="J5" s="41"/>
-      <c r="K5" s="88">
+      <c r="K5" s="87">
         <f t="shared" ref="K5:K9" si="1">COUNTA(C5:J5)-COUNTIF(C5:G5,"X")</f>
         <v>0</v>
       </c>
-      <c r="L5" s="89">
+      <c r="L5" s="88">
         <f t="shared" ref="L5:L16" si="2">COUNTIF(C5:J5,"X")</f>
         <v>0</v>
       </c>
-      <c r="M5" s="90" t="str">
+      <c r="M5" s="89" t="str">
         <f t="shared" ref="M5:M16" si="3">K5/COUNTA(C5:J5)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="N5" s="91" t="str">
+      <c r="N5" s="90" t="str">
         <f t="shared" ref="N5:N16" si="4">L5/COUNTA(C5:J5)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="O5" s="41"/>
     </row>
     <row r="6">
-      <c r="A6" s="86"/>
-      <c r="B6" s="86"/>
+      <c r="A6" s="85"/>
+      <c r="B6" s="85"/>
       <c r="C6" s="32"/>
       <c r="D6" s="32"/>
       <c r="E6" s="41"/>
@@ -20006,27 +19977,27 @@
       <c r="H6" s="41"/>
       <c r="I6" s="41"/>
       <c r="J6" s="41"/>
-      <c r="K6" s="88">
+      <c r="K6" s="87">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="L6" s="89">
+      <c r="L6" s="88">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M6" s="90" t="str">
+      <c r="M6" s="89" t="str">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="N6" s="91" t="str">
+      <c r="N6" s="90" t="str">
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="O6" s="41"/>
     </row>
     <row r="7">
-      <c r="A7" s="86"/>
-      <c r="B7" s="86"/>
+      <c r="A7" s="85"/>
+      <c r="B7" s="85"/>
       <c r="C7" s="32"/>
       <c r="D7" s="32"/>
       <c r="E7" s="41"/>
@@ -20035,27 +20006,27 @@
       <c r="H7" s="41"/>
       <c r="I7" s="41"/>
       <c r="J7" s="41"/>
-      <c r="K7" s="88">
+      <c r="K7" s="87">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="L7" s="89">
+      <c r="L7" s="88">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M7" s="90" t="str">
+      <c r="M7" s="89" t="str">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="N7" s="91" t="str">
+      <c r="N7" s="90" t="str">
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="O7" s="41"/>
     </row>
     <row r="8">
-      <c r="A8" s="86"/>
-      <c r="B8" s="86"/>
+      <c r="A8" s="85"/>
+      <c r="B8" s="85"/>
       <c r="C8" s="32"/>
       <c r="D8" s="32"/>
       <c r="E8" s="41"/>
@@ -20064,27 +20035,27 @@
       <c r="H8" s="41"/>
       <c r="I8" s="41"/>
       <c r="J8" s="41"/>
-      <c r="K8" s="88">
+      <c r="K8" s="87">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="L8" s="89">
+      <c r="L8" s="88">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M8" s="90" t="str">
+      <c r="M8" s="89" t="str">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="N8" s="91" t="str">
+      <c r="N8" s="90" t="str">
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="O8" s="41"/>
     </row>
     <row r="9">
-      <c r="A9" s="86"/>
-      <c r="B9" s="86"/>
+      <c r="A9" s="85"/>
+      <c r="B9" s="85"/>
       <c r="C9" s="32"/>
       <c r="D9" s="32"/>
       <c r="E9" s="41"/>
@@ -20093,27 +20064,27 @@
       <c r="H9" s="41"/>
       <c r="I9" s="41"/>
       <c r="J9" s="41"/>
-      <c r="K9" s="88">
+      <c r="K9" s="87">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="L9" s="89">
+      <c r="L9" s="88">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M9" s="90" t="str">
+      <c r="M9" s="89" t="str">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="N9" s="91" t="str">
+      <c r="N9" s="90" t="str">
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="O9" s="41"/>
     </row>
     <row r="10">
-      <c r="A10" s="86"/>
-      <c r="B10" s="86"/>
+      <c r="A10" s="85"/>
+      <c r="B10" s="85"/>
       <c r="C10" s="32"/>
       <c r="D10" s="32"/>
       <c r="E10" s="41"/>
@@ -20122,27 +20093,27 @@
       <c r="H10" s="41"/>
       <c r="I10" s="41"/>
       <c r="J10" s="41"/>
-      <c r="K10" s="88">
+      <c r="K10" s="87">
         <f>COUNTIF(C10:J10, "O")</f>
         <v>0</v>
       </c>
-      <c r="L10" s="89">
+      <c r="L10" s="88">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M10" s="90" t="str">
+      <c r="M10" s="89" t="str">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="N10" s="91" t="str">
+      <c r="N10" s="90" t="str">
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="O10" s="41"/>
     </row>
     <row r="11">
-      <c r="A11" s="86"/>
-      <c r="B11" s="87"/>
+      <c r="A11" s="85"/>
+      <c r="B11" s="86"/>
       <c r="C11" s="32"/>
       <c r="D11" s="32"/>
       <c r="E11" s="41"/>
@@ -20151,27 +20122,27 @@
       <c r="H11" s="41"/>
       <c r="I11" s="41"/>
       <c r="J11" s="41"/>
-      <c r="K11" s="88">
+      <c r="K11" s="87">
         <f t="shared" ref="K11:K16" si="5">COUNTA(C11:J11)-COUNTIF(C11:G11,"X")</f>
         <v>0</v>
       </c>
-      <c r="L11" s="89">
+      <c r="L11" s="88">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M11" s="90" t="str">
+      <c r="M11" s="89" t="str">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="N11" s="91" t="str">
+      <c r="N11" s="90" t="str">
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="O11" s="41"/>
     </row>
     <row r="12">
-      <c r="A12" s="86"/>
-      <c r="B12" s="86"/>
+      <c r="A12" s="85"/>
+      <c r="B12" s="85"/>
       <c r="C12" s="32"/>
       <c r="D12" s="32"/>
       <c r="E12" s="41"/>
@@ -20180,27 +20151,27 @@
       <c r="H12" s="41"/>
       <c r="I12" s="41"/>
       <c r="J12" s="41"/>
-      <c r="K12" s="88">
+      <c r="K12" s="87">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="L12" s="89">
+      <c r="L12" s="88">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M12" s="90" t="str">
+      <c r="M12" s="89" t="str">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="N12" s="91" t="str">
+      <c r="N12" s="90" t="str">
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="O12" s="41"/>
     </row>
     <row r="13">
-      <c r="A13" s="86"/>
-      <c r="B13" s="86"/>
+      <c r="A13" s="85"/>
+      <c r="B13" s="85"/>
       <c r="C13" s="41"/>
       <c r="D13" s="41"/>
       <c r="E13" s="41"/>
@@ -20209,27 +20180,27 @@
       <c r="H13" s="41"/>
       <c r="I13" s="41"/>
       <c r="J13" s="41"/>
-      <c r="K13" s="88">
+      <c r="K13" s="87">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="L13" s="89">
+      <c r="L13" s="88">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M13" s="90" t="str">
+      <c r="M13" s="89" t="str">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="N13" s="91" t="str">
+      <c r="N13" s="90" t="str">
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="O13" s="41"/>
     </row>
     <row r="14">
-      <c r="A14" s="86"/>
-      <c r="B14" s="86"/>
+      <c r="A14" s="85"/>
+      <c r="B14" s="85"/>
       <c r="C14" s="41"/>
       <c r="D14" s="41"/>
       <c r="E14" s="41"/>
@@ -20238,27 +20209,27 @@
       <c r="H14" s="41"/>
       <c r="I14" s="41"/>
       <c r="J14" s="41"/>
-      <c r="K14" s="88">
+      <c r="K14" s="87">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="L14" s="89">
+      <c r="L14" s="88">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M14" s="90" t="str">
+      <c r="M14" s="89" t="str">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="N14" s="91" t="str">
+      <c r="N14" s="90" t="str">
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="O14" s="41"/>
     </row>
     <row r="15">
-      <c r="A15" s="86"/>
-      <c r="B15" s="86"/>
+      <c r="A15" s="85"/>
+      <c r="B15" s="85"/>
       <c r="C15" s="41"/>
       <c r="D15" s="41"/>
       <c r="E15" s="41"/>
@@ -20267,27 +20238,27 @@
       <c r="H15" s="41"/>
       <c r="I15" s="41"/>
       <c r="J15" s="41"/>
-      <c r="K15" s="88">
+      <c r="K15" s="87">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="L15" s="89">
+      <c r="L15" s="88">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M15" s="90" t="str">
+      <c r="M15" s="89" t="str">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="N15" s="91" t="str">
+      <c r="N15" s="90" t="str">
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="O15" s="41"/>
     </row>
     <row r="16" ht="15.75" customHeight="1">
-      <c r="A16" s="86"/>
-      <c r="B16" s="86"/>
+      <c r="A16" s="85"/>
+      <c r="B16" s="85"/>
       <c r="C16" s="41"/>
       <c r="D16" s="41"/>
       <c r="E16" s="41"/>
@@ -20296,40 +20267,40 @@
       <c r="H16" s="41"/>
       <c r="I16" s="41"/>
       <c r="J16" s="41"/>
-      <c r="K16" s="88">
+      <c r="K16" s="87">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="L16" s="89">
+      <c r="L16" s="88">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M16" s="90" t="str">
+      <c r="M16" s="89" t="str">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="N16" s="91" t="str">
+      <c r="N16" s="90" t="str">
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
       <c r="O16" s="41"/>
     </row>
     <row r="18">
-      <c r="A18" s="92" t="s">
-        <v>38</v>
+      <c r="A18" s="91" t="s">
+        <v>47</v>
       </c>
-      <c r="B18" s="93" t="s">
-        <v>39</v>
+      <c r="B18" s="92" t="s">
+        <v>48</v>
       </c>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
     </row>
     <row r="19">
-      <c r="A19" s="94" t="s">
-        <v>40</v>
+      <c r="A19" s="93" t="s">
+        <v>49</v>
       </c>
-      <c r="B19" s="93" t="s">
-        <v>41</v>
+      <c r="B19" s="92" t="s">
+        <v>50</v>
       </c>
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
@@ -20337,9 +20308,9 @@
       <c r="F19" s="1"/>
     </row>
     <row r="20">
-      <c r="A20" s="95"/>
-      <c r="B20" s="93" t="s">
-        <v>42</v>
+      <c r="A20" s="94"/>
+      <c r="B20" s="92" t="s">
+        <v>51</v>
       </c>
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
@@ -20347,9 +20318,9 @@
       <c r="F20" s="1"/>
     </row>
     <row r="21">
-      <c r="A21" s="96"/>
-      <c r="B21" s="93" t="s">
-        <v>43</v>
+      <c r="A21" s="95"/>
+      <c r="B21" s="92" t="s">
+        <v>52</v>
       </c>
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>

</xml_diff>

<commit_message>
Updated class documents and months/days in spanish
Annoying .DS_Stor file keeps popping up
I have to deal with that later...
</commit_message>
<xml_diff>
--- a/class documents/roster.xlsx
+++ b/class documents/roster.xlsx
@@ -6,7 +6,7 @@
     <sheet state="visible" name="Class Roster" sheetId="1" r:id="rId4"/>
     <sheet state="visible" name="Student List" sheetId="2" r:id="rId5"/>
     <sheet state="visible" name="Demographic Data" sheetId="3" r:id="rId6"/>
-    <sheet state="visible" name="{Month} {Year}" sheetId="4" r:id="rId7"/>
+    <sheet state="visible" name="Month Year" sheetId="4" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="StudentName">#REF!</definedName>
@@ -30,7 +30,7 @@
         <color rgb="FFFFFFFF"/>
         <sz val="24.0"/>
       </rPr>
-      <t>Dev/Mission HQ 360 Valencia - {Month} {Year}</t>
+      <t>Dev/Mission HQ 360 Valencia - Month Year</t>
     </r>
     <r>
       <rPr>
@@ -48,7 +48,7 @@
     <t xml:space="preserve">START DATE </t>
   </si>
   <si>
-    <t>{Start}</t>
+    <t>Start</t>
   </si>
   <si>
     <t>INSTRUCTOR -  Jesus Arambula</t>
@@ -57,13 +57,13 @@
     <t>END DATE</t>
   </si>
   <si>
-    <t>{End}</t>
+    <t>End</t>
   </si>
   <si>
     <t>STUDENTS ENROLLED</t>
   </si>
   <si>
-    <t>{Day1} and {Day2} from 11:00 AM - 1:00 PM</t>
+    <t>Day1 and Day2 from 11:00 AM - 1:00 PM</t>
   </si>
   <si>
     <t xml:space="preserve"> </t>
@@ -115,7 +115,7 @@
         <color rgb="FFFFFFFF"/>
         <sz val="24.0"/>
       </rPr>
-      <t>Dev/Mission HQ 360 Valencia - {Month} {Year}</t>
+      <t>Dev/Mission HQ 360 Valencia - Month Year</t>
     </r>
     <r>
       <rPr>
@@ -142,13 +142,13 @@
     <t>GENDER</t>
   </si>
   <si>
-    <t>Starting Date</t>
+    <t>Month Year</t>
   </si>
   <si>
-    <t>{Day1}</t>
+    <t>Day1</t>
   </si>
   <si>
-    <t>{Day2}</t>
+    <t>Day2</t>
   </si>
   <si>
     <t>Present Days</t>
@@ -172,28 +172,28 @@
     <t xml:space="preserve">Last Name </t>
   </si>
   <si>
-    <t>{Date1}</t>
+    <t>Date1</t>
   </si>
   <si>
-    <t>{Date2}</t>
+    <t>Date2</t>
   </si>
   <si>
-    <t>{Date3}</t>
+    <t>Date3</t>
   </si>
   <si>
-    <t>{Date4}</t>
+    <t>Date4</t>
   </si>
   <si>
-    <t>{Date5}</t>
+    <t>Date5</t>
   </si>
   <si>
-    <t>{Date6}</t>
+    <t>Date6</t>
   </si>
   <si>
-    <t>{Date7}</t>
+    <t>Date7</t>
   </si>
   <si>
-    <t>{Date8}</t>
+    <t>Date8</t>
   </si>
   <si>
     <t>O</t>
@@ -223,7 +223,7 @@
     <numFmt numFmtId="165" formatCode="(###) ###-####"/>
     <numFmt numFmtId="166" formatCode="M/d/yyyy"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="16">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -263,12 +263,6 @@
     <font>
       <b/>
       <color theme="1"/>
-      <name val="Montserrat"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14.0"/>
-      <color rgb="FF333333"/>
       <name val="Montserrat"/>
     </font>
     <font>
@@ -579,7 +573,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="92">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
@@ -659,10 +653,31 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="12" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="12" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="12" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="12" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="12" fillId="0" fontId="6" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="12" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="12" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
     <xf borderId="12" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
@@ -670,22 +685,10 @@
     <xf borderId="12" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="12" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf borderId="12" fillId="0" fontId="6" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="12" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf borderId="12" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="12" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="12" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -745,16 +748,13 @@
     <xf borderId="12" fillId="4" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf borderId="12" fillId="4" fontId="6" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
     <xf borderId="12" fillId="6" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="12" fillId="4" fontId="6" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf borderId="12" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf borderId="12" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf borderId="12" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -763,31 +763,13 @@
     <xf borderId="12" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="12" fillId="4" fontId="1" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="12" fillId="4" fontId="1" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf borderId="12" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf borderId="12" fillId="6" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="12" fillId="6" fontId="6" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="12" fillId="6" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
     <xf borderId="0" fillId="6" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="12" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="12" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="16" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="16" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
     <xf borderId="17" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -796,13 +778,13 @@
     <xf borderId="18" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf borderId="19" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="19" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="20" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf borderId="12" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="12" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
     <xf borderId="21" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -811,52 +793,52 @@
     <xf borderId="22" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf borderId="12" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="12" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="bottom"/>
     </xf>
-    <xf borderId="23" fillId="7" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="23" fillId="7" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="23" fillId="8" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="23" fillId="8" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="23" fillId="9" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="23" fillId="9" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="23" fillId="10" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="23" fillId="10" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="23" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="12" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="12" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="24" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf borderId="12" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="12" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="25" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="25" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf borderId="12" fillId="7" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="12" fillId="7" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="right" vertical="bottom"/>
     </xf>
-    <xf borderId="12" fillId="8" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="12" fillId="8" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="right" vertical="bottom"/>
     </xf>
-    <xf borderId="12" fillId="9" fontId="13" numFmtId="10" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="12" fillId="9" fontId="12" numFmtId="10" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" vertical="bottom"/>
     </xf>
-    <xf borderId="12" fillId="10" fontId="13" numFmtId="10" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="12" fillId="10" fontId="12" numFmtId="10" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="11" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf borderId="0" fillId="12" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
@@ -974,7 +956,7 @@
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
+        <a:blip cstate="print" r:embed="rId3"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1460,263 +1442,305 @@
       <c r="H8" s="26"/>
       <c r="I8" s="26"/>
       <c r="J8" s="29"/>
-      <c r="K8" s="30"/>
+      <c r="K8" s="30">
+        <f t="shared" ref="K8:K21" si="1">DATEDIF(L8, TODAY(), "Y")</f>
+        <v>126</v>
+      </c>
       <c r="L8" s="31"/>
       <c r="M8" s="32"/>
-      <c r="N8" s="26"/>
+      <c r="N8" s="33"/>
       <c r="O8" s="20"/>
-      <c r="P8" s="33"/>
+      <c r="P8" s="34"/>
     </row>
     <row r="9" ht="21.0" customHeight="1">
       <c r="A9" s="1"/>
       <c r="B9" s="10"/>
-      <c r="C9" s="26"/>
-      <c r="D9" s="26"/>
-      <c r="E9" s="26"/>
-      <c r="F9" s="28"/>
-      <c r="G9" s="26"/>
-      <c r="H9" s="26"/>
-      <c r="I9" s="26"/>
-      <c r="J9" s="29"/>
-      <c r="K9" s="30"/>
-      <c r="L9" s="31"/>
+      <c r="C9" s="33"/>
+      <c r="D9" s="33"/>
+      <c r="E9" s="33"/>
+      <c r="F9" s="35"/>
+      <c r="G9" s="33"/>
+      <c r="H9" s="33"/>
+      <c r="I9" s="33"/>
+      <c r="J9" s="36"/>
+      <c r="K9" s="30">
+        <f t="shared" si="1"/>
+        <v>126</v>
+      </c>
+      <c r="L9" s="37"/>
       <c r="M9" s="32"/>
-      <c r="N9" s="26"/>
+      <c r="N9" s="33"/>
       <c r="O9" s="20"/>
       <c r="P9" s="1"/>
     </row>
     <row r="10" ht="21.0" customHeight="1">
       <c r="A10" s="1"/>
       <c r="B10" s="10"/>
-      <c r="C10" s="26"/>
-      <c r="D10" s="26"/>
-      <c r="E10" s="26"/>
-      <c r="F10" s="28"/>
-      <c r="G10" s="26"/>
-      <c r="H10" s="26"/>
-      <c r="I10" s="26"/>
-      <c r="J10" s="29"/>
-      <c r="K10" s="30"/>
-      <c r="L10" s="31"/>
+      <c r="C10" s="33"/>
+      <c r="D10" s="33"/>
+      <c r="E10" s="33"/>
+      <c r="F10" s="35"/>
+      <c r="G10" s="33"/>
+      <c r="H10" s="33"/>
+      <c r="I10" s="33"/>
+      <c r="J10" s="36"/>
+      <c r="K10" s="30">
+        <f t="shared" si="1"/>
+        <v>126</v>
+      </c>
+      <c r="L10" s="37"/>
       <c r="M10" s="32"/>
-      <c r="N10" s="26"/>
+      <c r="N10" s="33"/>
       <c r="O10" s="20"/>
-      <c r="P10" s="33"/>
+      <c r="P10" s="34"/>
     </row>
     <row r="11" ht="21.0" customHeight="1">
       <c r="A11" s="1"/>
       <c r="B11" s="10"/>
-      <c r="C11" s="26"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="28"/>
-      <c r="G11" s="26"/>
-      <c r="H11" s="26"/>
-      <c r="I11" s="26"/>
-      <c r="J11" s="29"/>
-      <c r="K11" s="30"/>
-      <c r="L11" s="31"/>
+      <c r="C11" s="33"/>
+      <c r="D11" s="33"/>
+      <c r="E11" s="33"/>
+      <c r="F11" s="35"/>
+      <c r="G11" s="33"/>
+      <c r="H11" s="33"/>
+      <c r="I11" s="33"/>
+      <c r="J11" s="36"/>
+      <c r="K11" s="30">
+        <f t="shared" si="1"/>
+        <v>126</v>
+      </c>
+      <c r="L11" s="37"/>
       <c r="M11" s="32"/>
-      <c r="N11" s="26"/>
+      <c r="N11" s="33"/>
       <c r="O11" s="20"/>
-      <c r="P11" s="33"/>
+      <c r="P11" s="34"/>
     </row>
     <row r="12" ht="21.0" customHeight="1">
       <c r="A12" s="1"/>
       <c r="B12" s="10"/>
-      <c r="C12" s="26"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="26"/>
-      <c r="F12" s="28"/>
-      <c r="G12" s="26"/>
-      <c r="H12" s="26"/>
-      <c r="I12" s="26"/>
-      <c r="J12" s="29"/>
-      <c r="K12" s="30"/>
-      <c r="L12" s="31"/>
-      <c r="M12" s="34"/>
-      <c r="N12" s="34"/>
+      <c r="C12" s="33"/>
+      <c r="D12" s="33"/>
+      <c r="E12" s="33"/>
+      <c r="F12" s="35"/>
+      <c r="G12" s="33"/>
+      <c r="H12" s="33"/>
+      <c r="I12" s="33"/>
+      <c r="J12" s="36"/>
+      <c r="K12" s="30">
+        <f t="shared" si="1"/>
+        <v>126</v>
+      </c>
+      <c r="L12" s="37"/>
+      <c r="M12" s="38"/>
+      <c r="N12" s="38"/>
       <c r="O12" s="20"/>
       <c r="P12" s="1"/>
     </row>
     <row r="13" ht="21.0" customHeight="1">
       <c r="A13" s="1"/>
       <c r="B13" s="10"/>
-      <c r="C13" s="26"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26"/>
-      <c r="F13" s="28"/>
-      <c r="G13" s="26"/>
-      <c r="H13" s="26"/>
-      <c r="I13" s="26"/>
-      <c r="J13" s="29"/>
-      <c r="K13" s="30"/>
-      <c r="L13" s="31"/>
+      <c r="C13" s="33"/>
+      <c r="D13" s="33"/>
+      <c r="E13" s="33"/>
+      <c r="F13" s="35"/>
+      <c r="G13" s="33"/>
+      <c r="H13" s="33"/>
+      <c r="I13" s="33"/>
+      <c r="J13" s="36"/>
+      <c r="K13" s="30">
+        <f t="shared" si="1"/>
+        <v>126</v>
+      </c>
+      <c r="L13" s="37"/>
       <c r="M13" s="32"/>
-      <c r="N13" s="26"/>
+      <c r="N13" s="33"/>
       <c r="O13" s="20"/>
       <c r="P13" s="1"/>
     </row>
     <row r="14" ht="21.0" customHeight="1">
       <c r="A14" s="1"/>
       <c r="B14" s="10"/>
-      <c r="C14" s="26"/>
-      <c r="D14" s="26"/>
-      <c r="E14" s="26"/>
-      <c r="F14" s="28"/>
-      <c r="G14" s="26"/>
-      <c r="H14" s="26"/>
-      <c r="I14" s="26"/>
-      <c r="J14" s="29"/>
-      <c r="K14" s="35"/>
-      <c r="L14" s="31"/>
+      <c r="C14" s="33"/>
+      <c r="D14" s="33"/>
+      <c r="E14" s="33"/>
+      <c r="F14" s="35"/>
+      <c r="G14" s="33"/>
+      <c r="H14" s="33"/>
+      <c r="I14" s="33"/>
+      <c r="J14" s="36"/>
+      <c r="K14" s="30">
+        <f t="shared" si="1"/>
+        <v>126</v>
+      </c>
+      <c r="L14" s="37"/>
       <c r="M14" s="32"/>
-      <c r="N14" s="26"/>
+      <c r="N14" s="33"/>
       <c r="O14" s="20"/>
       <c r="P14" s="1"/>
     </row>
     <row r="15" ht="21.0" customHeight="1">
       <c r="A15" s="1"/>
       <c r="B15" s="10"/>
-      <c r="C15" s="26"/>
-      <c r="D15" s="26"/>
-      <c r="E15" s="26"/>
-      <c r="F15" s="28"/>
-      <c r="G15" s="26"/>
-      <c r="H15" s="26"/>
-      <c r="I15" s="26"/>
-      <c r="J15" s="29"/>
-      <c r="K15" s="35"/>
-      <c r="L15" s="31"/>
+      <c r="C15" s="33"/>
+      <c r="D15" s="33"/>
+      <c r="E15" s="33"/>
+      <c r="F15" s="35"/>
+      <c r="G15" s="33"/>
+      <c r="H15" s="33"/>
+      <c r="I15" s="33"/>
+      <c r="J15" s="36"/>
+      <c r="K15" s="30">
+        <f t="shared" si="1"/>
+        <v>126</v>
+      </c>
+      <c r="L15" s="37"/>
       <c r="M15" s="32"/>
-      <c r="N15" s="26"/>
+      <c r="N15" s="33"/>
       <c r="O15" s="20"/>
       <c r="P15" s="1"/>
     </row>
     <row r="16" ht="21.0" customHeight="1">
       <c r="A16" s="1"/>
       <c r="B16" s="10"/>
-      <c r="C16" s="26"/>
-      <c r="D16" s="26"/>
-      <c r="E16" s="26"/>
-      <c r="F16" s="28"/>
-      <c r="G16" s="26"/>
-      <c r="H16" s="26"/>
-      <c r="I16" s="26"/>
-      <c r="J16" s="29"/>
-      <c r="K16" s="35"/>
-      <c r="L16" s="31"/>
+      <c r="C16" s="33"/>
+      <c r="D16" s="33"/>
+      <c r="E16" s="33"/>
+      <c r="F16" s="35"/>
+      <c r="G16" s="33"/>
+      <c r="H16" s="33"/>
+      <c r="I16" s="33"/>
+      <c r="J16" s="36"/>
+      <c r="K16" s="30">
+        <f t="shared" si="1"/>
+        <v>126</v>
+      </c>
+      <c r="L16" s="37"/>
       <c r="M16" s="32"/>
-      <c r="N16" s="26"/>
+      <c r="N16" s="33"/>
       <c r="O16" s="20"/>
       <c r="P16" s="1"/>
     </row>
     <row r="17" ht="21.0" customHeight="1">
       <c r="A17" s="1"/>
       <c r="B17" s="10"/>
-      <c r="C17" s="36"/>
-      <c r="D17" s="36"/>
+      <c r="C17" s="39"/>
+      <c r="D17" s="39"/>
       <c r="E17" s="32"/>
-      <c r="F17" s="37"/>
+      <c r="F17" s="40"/>
       <c r="G17" s="32"/>
       <c r="H17" s="32"/>
       <c r="I17" s="32"/>
-      <c r="J17" s="38"/>
-      <c r="K17" s="35"/>
-      <c r="L17" s="39"/>
-      <c r="M17" s="40"/>
-      <c r="N17" s="40"/>
+      <c r="J17" s="41"/>
+      <c r="K17" s="30">
+        <f t="shared" si="1"/>
+        <v>126</v>
+      </c>
+      <c r="L17" s="42"/>
+      <c r="M17" s="43"/>
+      <c r="N17" s="43"/>
       <c r="O17" s="20"/>
       <c r="P17" s="1"/>
     </row>
     <row r="18" ht="21.0" customHeight="1">
       <c r="A18" s="1"/>
       <c r="B18" s="10"/>
-      <c r="C18" s="36"/>
-      <c r="D18" s="36"/>
+      <c r="C18" s="39"/>
+      <c r="D18" s="39"/>
       <c r="E18" s="32"/>
-      <c r="F18" s="37"/>
+      <c r="F18" s="40"/>
       <c r="G18" s="32"/>
       <c r="H18" s="32"/>
       <c r="I18" s="32"/>
-      <c r="J18" s="38"/>
-      <c r="K18" s="35"/>
-      <c r="L18" s="39"/>
-      <c r="M18" s="40"/>
-      <c r="N18" s="40"/>
+      <c r="J18" s="41"/>
+      <c r="K18" s="30">
+        <f t="shared" si="1"/>
+        <v>126</v>
+      </c>
+      <c r="L18" s="42"/>
+      <c r="M18" s="43"/>
+      <c r="N18" s="43"/>
       <c r="O18" s="20"/>
-      <c r="P18" s="33"/>
+      <c r="P18" s="34"/>
     </row>
     <row r="19" ht="21.0" customHeight="1">
       <c r="A19" s="1"/>
       <c r="B19" s="10"/>
-      <c r="C19" s="36"/>
-      <c r="D19" s="36"/>
+      <c r="C19" s="39"/>
+      <c r="D19" s="39"/>
       <c r="E19" s="32"/>
-      <c r="F19" s="37"/>
+      <c r="F19" s="40"/>
       <c r="G19" s="32"/>
       <c r="H19" s="32"/>
       <c r="I19" s="32"/>
-      <c r="J19" s="38"/>
-      <c r="K19" s="35"/>
-      <c r="L19" s="39"/>
-      <c r="M19" s="41"/>
-      <c r="N19" s="41"/>
+      <c r="J19" s="41"/>
+      <c r="K19" s="30">
+        <f t="shared" si="1"/>
+        <v>126</v>
+      </c>
+      <c r="L19" s="42"/>
+      <c r="M19" s="44"/>
+      <c r="N19" s="44"/>
       <c r="O19" s="20"/>
-      <c r="P19" s="33"/>
+      <c r="P19" s="34"/>
     </row>
     <row r="20" ht="21.0" customHeight="1">
       <c r="A20" s="1"/>
       <c r="B20" s="10"/>
-      <c r="C20" s="40"/>
-      <c r="D20" s="40"/>
-      <c r="E20" s="37"/>
-      <c r="F20" s="37"/>
+      <c r="C20" s="43"/>
+      <c r="D20" s="43"/>
+      <c r="E20" s="40"/>
+      <c r="F20" s="40"/>
       <c r="G20" s="32"/>
       <c r="H20" s="32"/>
       <c r="I20" s="32"/>
-      <c r="J20" s="38"/>
-      <c r="K20" s="35"/>
-      <c r="L20" s="42"/>
-      <c r="M20" s="41"/>
-      <c r="N20" s="41"/>
+      <c r="J20" s="41"/>
+      <c r="K20" s="30">
+        <f t="shared" si="1"/>
+        <v>126</v>
+      </c>
+      <c r="L20" s="45"/>
+      <c r="M20" s="44"/>
+      <c r="N20" s="44"/>
       <c r="O20" s="20"/>
-      <c r="P20" s="33"/>
+      <c r="P20" s="34"/>
     </row>
     <row r="21" ht="21.0" customHeight="1">
       <c r="A21" s="1"/>
       <c r="B21" s="10"/>
-      <c r="C21" s="40"/>
-      <c r="D21" s="40"/>
-      <c r="E21" s="37"/>
-      <c r="F21" s="37"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="40"/>
+      <c r="F21" s="40"/>
       <c r="G21" s="32"/>
       <c r="H21" s="32"/>
       <c r="I21" s="32"/>
-      <c r="J21" s="38"/>
-      <c r="K21" s="35"/>
-      <c r="L21" s="42"/>
-      <c r="M21" s="41"/>
-      <c r="N21" s="41"/>
+      <c r="J21" s="41"/>
+      <c r="K21" s="30">
+        <f t="shared" si="1"/>
+        <v>126</v>
+      </c>
+      <c r="L21" s="45"/>
+      <c r="M21" s="44"/>
+      <c r="N21" s="44"/>
       <c r="O21" s="20"/>
-      <c r="P21" s="33"/>
+      <c r="P21" s="34"/>
     </row>
     <row r="22" ht="21.0" customHeight="1">
       <c r="A22" s="1"/>
-      <c r="B22" s="43"/>
-      <c r="C22" s="44"/>
-      <c r="D22" s="44"/>
-      <c r="E22" s="45"/>
-      <c r="F22" s="45"/>
-      <c r="G22" s="46"/>
-      <c r="H22" s="46"/>
-      <c r="I22" s="46"/>
-      <c r="J22" s="47"/>
-      <c r="K22" s="44"/>
-      <c r="L22" s="44"/>
-      <c r="M22" s="44"/>
-      <c r="N22" s="44"/>
-      <c r="O22" s="48"/>
+      <c r="B22" s="46"/>
+      <c r="C22" s="47"/>
+      <c r="D22" s="47"/>
+      <c r="E22" s="48"/>
+      <c r="F22" s="48"/>
+      <c r="G22" s="49"/>
+      <c r="H22" s="49"/>
+      <c r="I22" s="49"/>
+      <c r="J22" s="50"/>
+      <c r="K22" s="47"/>
+      <c r="L22" s="47"/>
+      <c r="M22" s="47"/>
+      <c r="N22" s="47"/>
+      <c r="O22" s="51"/>
       <c r="P22" s="1"/>
     </row>
     <row r="23" ht="21.0" customHeight="1">
@@ -19307,11 +19331,11 @@
     </row>
   </sheetData>
   <mergeCells count="5">
+    <mergeCell ref="E2:J2"/>
     <mergeCell ref="F3:I5"/>
     <mergeCell ref="J3:K3"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="J5:L5"/>
-    <mergeCell ref="E2:J2"/>
   </mergeCells>
   <printOptions gridLines="1" horizontalCentered="1"/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
@@ -19351,285 +19375,465 @@
       <c r="J2" s="8"/>
     </row>
     <row r="4">
-      <c r="A4" s="49" t="s">
+      <c r="A4" s="52" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="49" t="s">
+      <c r="B4" s="52" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="49" t="s">
+      <c r="C4" s="52" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="49" t="s">
+      <c r="D4" s="52" t="s">
         <v>26</v>
       </c>
-      <c r="E4" s="49" t="s">
+      <c r="E4" s="52" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="49" t="s">
+      <c r="F4" s="52" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="49" t="s">
+      <c r="G4" s="52" t="s">
         <v>16</v>
       </c>
-      <c r="H4" s="49" t="s">
+      <c r="H4" s="52" t="s">
         <v>17</v>
       </c>
-      <c r="I4" s="49" t="s">
+      <c r="I4" s="52" t="s">
         <v>27</v>
       </c>
-      <c r="J4" s="49" t="s">
+      <c r="J4" s="52" t="s">
         <v>28</v>
       </c>
-      <c r="K4" s="50" t="s">
+      <c r="K4" s="53" t="s">
         <v>19</v>
       </c>
-      <c r="L4" s="49" t="s">
+      <c r="L4" s="52" t="s">
         <v>18</v>
       </c>
-      <c r="M4" s="49" t="s">
+      <c r="M4" s="52" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="51">
+      <c r="A5" s="54">
         <v>1.0</v>
       </c>
-      <c r="B5" s="52"/>
-      <c r="C5" s="53"/>
-      <c r="D5" s="52"/>
-      <c r="E5" s="52"/>
-      <c r="F5" s="52"/>
-      <c r="G5" s="26"/>
-      <c r="H5" s="54"/>
+      <c r="B5" s="55" t="str">
+        <f t="array" ref="B5:C5">'Class Roster'!C8:D8</f>
+        <v/>
+      </c>
+      <c r="C5" s="56"/>
+      <c r="D5" s="55" t="str">
+        <f t="array" ref="D5:G5">'Class Roster'!F8:I8</f>
+        <v/>
+      </c>
+      <c r="E5" s="55"/>
+      <c r="F5" s="55"/>
+      <c r="G5" s="55"/>
+      <c r="H5" s="57" t="str">
+        <f>'Class Roster'!J8</f>
+        <v/>
+      </c>
       <c r="I5" s="55"/>
       <c r="J5" s="55"/>
-      <c r="K5" s="56"/>
-      <c r="L5" s="55">
+      <c r="K5" s="58" t="str">
+        <f>'Class Roster'!L8</f>
+        <v/>
+      </c>
+      <c r="L5" s="59">
         <f t="shared" ref="L5:L16" si="1">DATEDIF(K5, TODAY(), "Y")</f>
         <v>126</v>
       </c>
-      <c r="M5" s="57"/>
+      <c r="M5" s="60" t="str">
+        <f>'Class Roster'!E8</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="51">
+      <c r="A6" s="54">
         <v>2.0</v>
       </c>
-      <c r="B6" s="26"/>
-      <c r="C6" s="26"/>
-      <c r="D6" s="26"/>
-      <c r="E6" s="26"/>
-      <c r="F6" s="26"/>
-      <c r="G6" s="26"/>
-      <c r="H6" s="29"/>
+      <c r="B6" s="55" t="str">
+        <f t="array" ref="B6:C6">'Class Roster'!C9:D9</f>
+        <v/>
+      </c>
+      <c r="C6" s="33"/>
+      <c r="D6" s="55" t="str">
+        <f t="array" ref="D6:G6">'Class Roster'!F9:I9</f>
+        <v/>
+      </c>
+      <c r="E6" s="55"/>
+      <c r="F6" s="55"/>
+      <c r="G6" s="55"/>
+      <c r="H6" s="57" t="str">
+        <f>'Class Roster'!J9</f>
+        <v/>
+      </c>
       <c r="I6" s="55"/>
       <c r="J6" s="55"/>
-      <c r="K6" s="31"/>
-      <c r="L6" s="55">
+      <c r="K6" s="58" t="str">
+        <f>'Class Roster'!L9</f>
+        <v/>
+      </c>
+      <c r="L6" s="59">
         <f t="shared" si="1"/>
         <v>126</v>
       </c>
-      <c r="M6" s="57"/>
+      <c r="M6" s="60" t="str">
+        <f>'Class Roster'!E9</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="51">
+      <c r="A7" s="54">
         <v>3.0</v>
       </c>
-      <c r="B7" s="52"/>
-      <c r="C7" s="52"/>
-      <c r="D7" s="52"/>
-      <c r="E7" s="52"/>
-      <c r="F7" s="52"/>
-      <c r="G7" s="26"/>
-      <c r="H7" s="54"/>
+      <c r="B7" s="55" t="str">
+        <f t="array" ref="B7:C7">'Class Roster'!C10:D10</f>
+        <v/>
+      </c>
+      <c r="C7" s="55"/>
+      <c r="D7" s="55" t="str">
+        <f t="array" ref="D7:G7">'Class Roster'!F10:I10</f>
+        <v/>
+      </c>
+      <c r="E7" s="55"/>
+      <c r="F7" s="55"/>
+      <c r="G7" s="55"/>
+      <c r="H7" s="57" t="str">
+        <f>'Class Roster'!J10</f>
+        <v/>
+      </c>
       <c r="I7" s="55"/>
       <c r="J7" s="55"/>
-      <c r="K7" s="56"/>
-      <c r="L7" s="55">
+      <c r="K7" s="58" t="str">
+        <f>'Class Roster'!L10</f>
+        <v/>
+      </c>
+      <c r="L7" s="59">
         <f t="shared" si="1"/>
         <v>126</v>
       </c>
-      <c r="M7" s="58"/>
+      <c r="M7" s="60" t="str">
+        <f>'Class Roster'!E10</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="51">
+      <c r="A8" s="54">
         <v>4.0</v>
       </c>
-      <c r="B8" s="52"/>
-      <c r="C8" s="52"/>
-      <c r="D8" s="52"/>
-      <c r="E8" s="52"/>
-      <c r="F8" s="52"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="54"/>
+      <c r="B8" s="55" t="str">
+        <f t="array" ref="B8:C8">'Class Roster'!C11:D11</f>
+        <v/>
+      </c>
+      <c r="C8" s="55"/>
+      <c r="D8" s="55" t="str">
+        <f t="array" ref="D8:G8">'Class Roster'!F11:I11</f>
+        <v/>
+      </c>
+      <c r="E8" s="55"/>
+      <c r="F8" s="55"/>
+      <c r="G8" s="55"/>
+      <c r="H8" s="57" t="str">
+        <f>'Class Roster'!J11</f>
+        <v/>
+      </c>
       <c r="I8" s="55"/>
       <c r="J8" s="55"/>
-      <c r="K8" s="56"/>
-      <c r="L8" s="55">
+      <c r="K8" s="58" t="str">
+        <f>'Class Roster'!L11</f>
+        <v/>
+      </c>
+      <c r="L8" s="59">
         <f t="shared" si="1"/>
         <v>126</v>
       </c>
-      <c r="M8" s="58"/>
+      <c r="M8" s="60" t="str">
+        <f>'Class Roster'!E11</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="51">
+      <c r="A9" s="54">
         <v>5.0</v>
       </c>
-      <c r="B9" s="26"/>
-      <c r="C9" s="26"/>
-      <c r="D9" s="26"/>
-      <c r="E9" s="26"/>
-      <c r="F9" s="26"/>
-      <c r="G9" s="26"/>
-      <c r="H9" s="29"/>
+      <c r="B9" s="55" t="str">
+        <f t="array" ref="B9:C9">'Class Roster'!C12:D12</f>
+        <v/>
+      </c>
+      <c r="C9" s="33"/>
+      <c r="D9" s="55" t="str">
+        <f t="array" ref="D9:G9">'Class Roster'!F12:I12</f>
+        <v/>
+      </c>
+      <c r="E9" s="55"/>
+      <c r="F9" s="55"/>
+      <c r="G9" s="55"/>
+      <c r="H9" s="57" t="str">
+        <f>'Class Roster'!J12</f>
+        <v/>
+      </c>
       <c r="I9" s="55"/>
       <c r="J9" s="55"/>
-      <c r="K9" s="31"/>
-      <c r="L9" s="55">
+      <c r="K9" s="58" t="str">
+        <f>'Class Roster'!L12</f>
+        <v/>
+      </c>
+      <c r="L9" s="59">
         <f t="shared" si="1"/>
         <v>126</v>
       </c>
-      <c r="M9" s="41"/>
+      <c r="M9" s="60" t="str">
+        <f>'Class Roster'!E12</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="51">
+      <c r="A10" s="54">
         <v>6.0</v>
       </c>
-      <c r="B10" s="26"/>
-      <c r="C10" s="26"/>
-      <c r="D10" s="26"/>
-      <c r="E10" s="26"/>
-      <c r="F10" s="26"/>
-      <c r="G10" s="26"/>
-      <c r="H10" s="29"/>
+      <c r="B10" s="55" t="str">
+        <f t="array" ref="B10:C10">'Class Roster'!C13:D13</f>
+        <v/>
+      </c>
+      <c r="C10" s="33"/>
+      <c r="D10" s="55" t="str">
+        <f t="array" ref="D10:G10">'Class Roster'!F13:I13</f>
+        <v/>
+      </c>
+      <c r="E10" s="55"/>
+      <c r="F10" s="55"/>
+      <c r="G10" s="55"/>
+      <c r="H10" s="57" t="str">
+        <f>'Class Roster'!J13</f>
+        <v/>
+      </c>
       <c r="I10" s="55"/>
       <c r="J10" s="55"/>
-      <c r="K10" s="31"/>
-      <c r="L10" s="55">
+      <c r="K10" s="58" t="str">
+        <f>'Class Roster'!L13</f>
+        <v/>
+      </c>
+      <c r="L10" s="59">
         <f t="shared" si="1"/>
         <v>126</v>
       </c>
-      <c r="M10" s="57"/>
+      <c r="M10" s="60" t="str">
+        <f>'Class Roster'!E13</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="51">
+      <c r="A11" s="54">
         <v>7.0</v>
       </c>
-      <c r="B11" s="59"/>
-      <c r="C11" s="59"/>
-      <c r="D11" s="60"/>
-      <c r="E11" s="60"/>
-      <c r="F11" s="60"/>
-      <c r="G11" s="32"/>
-      <c r="H11" s="61"/>
+      <c r="B11" s="55" t="str">
+        <f t="array" ref="B11:C11">'Class Roster'!C14:D14</f>
+        <v/>
+      </c>
+      <c r="C11" s="61"/>
+      <c r="D11" s="55" t="str">
+        <f t="array" ref="D11:G11">'Class Roster'!F14:I14</f>
+        <v/>
+      </c>
+      <c r="E11" s="62"/>
+      <c r="F11" s="62"/>
+      <c r="G11" s="62"/>
+      <c r="H11" s="57" t="str">
+        <f>'Class Roster'!J14</f>
+        <v/>
+      </c>
       <c r="I11" s="55"/>
       <c r="J11" s="55"/>
-      <c r="K11" s="62"/>
-      <c r="L11" s="55">
+      <c r="K11" s="58" t="str">
+        <f>'Class Roster'!L14</f>
+        <v/>
+      </c>
+      <c r="L11" s="59">
         <f t="shared" si="1"/>
         <v>126</v>
       </c>
-      <c r="M11" s="63"/>
+      <c r="M11" s="60" t="str">
+        <f>'Class Roster'!E14</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="51">
+      <c r="A12" s="54">
         <v>8.0</v>
       </c>
-      <c r="B12" s="59"/>
-      <c r="C12" s="59"/>
-      <c r="D12" s="60"/>
-      <c r="E12" s="60"/>
-      <c r="F12" s="60"/>
-      <c r="G12" s="32"/>
-      <c r="H12" s="61"/>
+      <c r="B12" s="55" t="str">
+        <f t="array" ref="B12:C12">'Class Roster'!C15:D15</f>
+        <v/>
+      </c>
+      <c r="C12" s="61"/>
+      <c r="D12" s="55" t="str">
+        <f t="array" ref="D12:G12">'Class Roster'!F15:I15</f>
+        <v/>
+      </c>
+      <c r="E12" s="62"/>
+      <c r="F12" s="62"/>
+      <c r="G12" s="62"/>
+      <c r="H12" s="57" t="str">
+        <f>'Class Roster'!J15</f>
+        <v/>
+      </c>
       <c r="I12" s="55"/>
       <c r="J12" s="55"/>
-      <c r="K12" s="62"/>
-      <c r="L12" s="55">
+      <c r="K12" s="58" t="str">
+        <f>'Class Roster'!L15</f>
+        <v/>
+      </c>
+      <c r="L12" s="59">
         <f t="shared" si="1"/>
         <v>126</v>
       </c>
-      <c r="M12" s="63"/>
+      <c r="M12" s="60" t="str">
+        <f>'Class Roster'!E15</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="51">
+      <c r="A13" s="54">
         <v>9.0</v>
       </c>
-      <c r="B13" s="55"/>
+      <c r="B13" s="55" t="str">
+        <f t="array" ref="B13:C13">'Class Roster'!C16:D16</f>
+        <v/>
+      </c>
       <c r="C13" s="55"/>
-      <c r="D13" s="55"/>
+      <c r="D13" s="55" t="str">
+        <f t="array" ref="D13:G13">'Class Roster'!F16:I16</f>
+        <v/>
+      </c>
       <c r="E13" s="55"/>
       <c r="F13" s="55"/>
       <c r="G13" s="55"/>
-      <c r="H13" s="64"/>
+      <c r="H13" s="57" t="str">
+        <f>'Class Roster'!J16</f>
+        <v/>
+      </c>
       <c r="I13" s="55"/>
       <c r="J13" s="55"/>
-      <c r="K13" s="65"/>
-      <c r="L13" s="55">
+      <c r="K13" s="58" t="str">
+        <f>'Class Roster'!L16</f>
+        <v/>
+      </c>
+      <c r="L13" s="59">
         <f t="shared" si="1"/>
         <v>126</v>
       </c>
-      <c r="M13" s="66"/>
+      <c r="M13" s="60" t="str">
+        <f>'Class Roster'!E16</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="51">
+      <c r="A14" s="54">
         <v>10.0</v>
       </c>
-      <c r="B14" s="55"/>
+      <c r="B14" s="55" t="str">
+        <f t="array" ref="B14:C14">'Class Roster'!C17:D17</f>
+        <v/>
+      </c>
       <c r="C14" s="55"/>
-      <c r="D14" s="55"/>
+      <c r="D14" s="55" t="str">
+        <f t="array" ref="D14:G14">'Class Roster'!F17:I17</f>
+        <v/>
+      </c>
       <c r="E14" s="55"/>
       <c r="F14" s="55"/>
       <c r="G14" s="55"/>
-      <c r="H14" s="64"/>
+      <c r="H14" s="57" t="str">
+        <f>'Class Roster'!J17</f>
+        <v/>
+      </c>
       <c r="I14" s="55"/>
       <c r="J14" s="55"/>
-      <c r="K14" s="65"/>
-      <c r="L14" s="55">
+      <c r="K14" s="58" t="str">
+        <f>'Class Roster'!L17</f>
+        <v/>
+      </c>
+      <c r="L14" s="59">
         <f t="shared" si="1"/>
         <v>126</v>
       </c>
-      <c r="M14" s="66"/>
+      <c r="M14" s="60" t="str">
+        <f>'Class Roster'!E17</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="51">
+      <c r="A15" s="54">
         <v>11.0</v>
       </c>
-      <c r="B15" s="55"/>
+      <c r="B15" s="55" t="str">
+        <f t="array" ref="B15:C15">'Class Roster'!C18:D18</f>
+        <v/>
+      </c>
       <c r="C15" s="55"/>
-      <c r="D15" s="55"/>
+      <c r="D15" s="55" t="str">
+        <f t="array" ref="D15:G15">'Class Roster'!F18:I18</f>
+        <v/>
+      </c>
       <c r="E15" s="55"/>
       <c r="F15" s="55"/>
       <c r="G15" s="55"/>
-      <c r="H15" s="64"/>
+      <c r="H15" s="57" t="str">
+        <f>'Class Roster'!J18</f>
+        <v/>
+      </c>
       <c r="I15" s="55"/>
       <c r="J15" s="55"/>
-      <c r="K15" s="65"/>
-      <c r="L15" s="55">
+      <c r="K15" s="58" t="str">
+        <f>'Class Roster'!L18</f>
+        <v/>
+      </c>
+      <c r="L15" s="59">
         <f t="shared" si="1"/>
         <v>126</v>
       </c>
-      <c r="M15" s="66"/>
+      <c r="M15" s="60" t="str">
+        <f>'Class Roster'!E18</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="51">
+      <c r="A16" s="54">
         <v>12.0</v>
       </c>
-      <c r="B16" s="55"/>
+      <c r="B16" s="55" t="str">
+        <f t="array" ref="B16:C16">'Class Roster'!C19:D19</f>
+        <v/>
+      </c>
       <c r="C16" s="55"/>
-      <c r="D16" s="55"/>
+      <c r="D16" s="55" t="str">
+        <f t="array" ref="D16:G16">'Class Roster'!F19:I19</f>
+        <v/>
+      </c>
       <c r="E16" s="55"/>
       <c r="F16" s="55"/>
       <c r="G16" s="55"/>
-      <c r="H16" s="64"/>
+      <c r="H16" s="57" t="str">
+        <f>'Class Roster'!J19</f>
+        <v/>
+      </c>
       <c r="I16" s="55"/>
       <c r="J16" s="55"/>
-      <c r="K16" s="65"/>
-      <c r="L16" s="55">
+      <c r="K16" s="58" t="str">
+        <f>'Class Roster'!L19</f>
+        <v/>
+      </c>
+      <c r="L16" s="59">
         <f t="shared" si="1"/>
         <v>126</v>
       </c>
-      <c r="M16" s="66"/>
+      <c r="M16" s="60" t="str">
+        <f>'Class Roster'!E19</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -19652,150 +19856,294 @@
   </cols>
   <sheetData>
     <row r="3">
-      <c r="B3" s="49" t="s">
+      <c r="B3" s="52" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="49" t="s">
+      <c r="C3" s="52" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="49" t="s">
+      <c r="D3" s="52" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="49" t="s">
+      <c r="E3" s="52" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="49" t="s">
+      <c r="F3" s="52" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="49" t="s">
+      <c r="G3" s="52" t="s">
         <v>27</v>
       </c>
-      <c r="H3" s="49" t="s">
+      <c r="H3" s="52" t="s">
         <v>28</v>
       </c>
-      <c r="I3" s="49" t="s">
+      <c r="I3" s="52" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="55"/>
-      <c r="C4" s="67"/>
-      <c r="D4" s="55"/>
-      <c r="E4" s="55"/>
-      <c r="F4" s="55"/>
-      <c r="G4" s="55"/>
-      <c r="H4" s="55"/>
-      <c r="I4" s="55"/>
+      <c r="B4" s="59" t="str">
+        <f t="array" ref="B4:C4">'Class Roster'!C8:D8</f>
+        <v/>
+      </c>
+      <c r="C4" s="63"/>
+      <c r="D4" s="59" t="str">
+        <f t="array" ref="D4:F4">'Class Roster'!G8:I8</f>
+        <v/>
+      </c>
+      <c r="E4" s="59"/>
+      <c r="F4" s="59"/>
+      <c r="G4" s="59" t="str">
+        <f t="array" ref="G4:H4">'Student List'!I5:J5</f>
+        <v/>
+      </c>
+      <c r="H4" s="59"/>
+      <c r="I4" s="59">
+        <f>'Class Roster'!K8</f>
+        <v>126</v>
+      </c>
     </row>
     <row r="5">
-      <c r="B5" s="55"/>
-      <c r="C5" s="55"/>
-      <c r="D5" s="55"/>
-      <c r="E5" s="55"/>
-      <c r="F5" s="55"/>
-      <c r="G5" s="55"/>
-      <c r="H5" s="55"/>
-      <c r="I5" s="55"/>
+      <c r="B5" s="59" t="str">
+        <f t="array" ref="B5:C5">'Class Roster'!C9:D9</f>
+        <v/>
+      </c>
+      <c r="C5" s="59"/>
+      <c r="D5" s="59" t="str">
+        <f t="array" ref="D5:F5">'Class Roster'!G9:I9</f>
+        <v/>
+      </c>
+      <c r="E5" s="59"/>
+      <c r="F5" s="59"/>
+      <c r="G5" s="59" t="str">
+        <f t="array" ref="G5:H5">'Student List'!I6:J6</f>
+        <v/>
+      </c>
+      <c r="H5" s="59"/>
+      <c r="I5" s="59">
+        <f>'Class Roster'!K9</f>
+        <v>126</v>
+      </c>
     </row>
     <row r="6">
-      <c r="B6" s="55"/>
-      <c r="C6" s="55"/>
-      <c r="D6" s="55"/>
-      <c r="E6" s="55"/>
-      <c r="F6" s="55"/>
-      <c r="G6" s="55"/>
-      <c r="H6" s="55"/>
-      <c r="I6" s="55"/>
+      <c r="B6" s="59" t="str">
+        <f t="array" ref="B6:C6">'Class Roster'!C10:D10</f>
+        <v/>
+      </c>
+      <c r="C6" s="59"/>
+      <c r="D6" s="59" t="str">
+        <f t="array" ref="D6:F6">'Class Roster'!G10:I10</f>
+        <v/>
+      </c>
+      <c r="E6" s="59"/>
+      <c r="F6" s="59"/>
+      <c r="G6" s="59" t="str">
+        <f t="array" ref="G6:H6">'Student List'!I7:J7</f>
+        <v/>
+      </c>
+      <c r="H6" s="59"/>
+      <c r="I6" s="59">
+        <f>'Class Roster'!K10</f>
+        <v>126</v>
+      </c>
     </row>
     <row r="7">
-      <c r="B7" s="55"/>
-      <c r="C7" s="55"/>
-      <c r="D7" s="55"/>
-      <c r="E7" s="55"/>
-      <c r="F7" s="55"/>
-      <c r="G7" s="55"/>
-      <c r="H7" s="55"/>
-      <c r="I7" s="55"/>
+      <c r="B7" s="59" t="str">
+        <f t="array" ref="B7:C7">'Class Roster'!C11:D11</f>
+        <v/>
+      </c>
+      <c r="C7" s="59"/>
+      <c r="D7" s="59" t="str">
+        <f t="array" ref="D7:F7">'Class Roster'!G11:I11</f>
+        <v/>
+      </c>
+      <c r="E7" s="59"/>
+      <c r="F7" s="59"/>
+      <c r="G7" s="59" t="str">
+        <f t="array" ref="G7:H7">'Student List'!I8:J8</f>
+        <v/>
+      </c>
+      <c r="H7" s="59"/>
+      <c r="I7" s="59">
+        <f>'Class Roster'!K11</f>
+        <v>126</v>
+      </c>
     </row>
     <row r="8">
-      <c r="B8" s="55"/>
-      <c r="C8" s="55"/>
-      <c r="D8" s="55"/>
-      <c r="E8" s="55"/>
-      <c r="F8" s="55"/>
-      <c r="G8" s="55"/>
-      <c r="H8" s="55"/>
-      <c r="I8" s="55"/>
+      <c r="B8" s="59" t="str">
+        <f t="array" ref="B8:C8">'Class Roster'!C12:D12</f>
+        <v/>
+      </c>
+      <c r="C8" s="59"/>
+      <c r="D8" s="59" t="str">
+        <f t="array" ref="D8:F8">'Class Roster'!G12:I12</f>
+        <v/>
+      </c>
+      <c r="E8" s="59"/>
+      <c r="F8" s="59"/>
+      <c r="G8" s="59" t="str">
+        <f t="array" ref="G8:H8">'Student List'!I9:J9</f>
+        <v/>
+      </c>
+      <c r="H8" s="59"/>
+      <c r="I8" s="59">
+        <f>'Class Roster'!K12</f>
+        <v>126</v>
+      </c>
     </row>
     <row r="9">
-      <c r="B9" s="55"/>
-      <c r="C9" s="55"/>
-      <c r="D9" s="55"/>
-      <c r="E9" s="55"/>
-      <c r="F9" s="55"/>
-      <c r="G9" s="55"/>
-      <c r="H9" s="55"/>
-      <c r="I9" s="55"/>
+      <c r="B9" s="59" t="str">
+        <f t="array" ref="B9:C9">'Class Roster'!C13:D13</f>
+        <v/>
+      </c>
+      <c r="C9" s="59"/>
+      <c r="D9" s="59" t="str">
+        <f t="array" ref="D9:F9">'Class Roster'!G13:I13</f>
+        <v/>
+      </c>
+      <c r="E9" s="59"/>
+      <c r="F9" s="59"/>
+      <c r="G9" s="59" t="str">
+        <f t="array" ref="G9:H9">'Student List'!I10:J10</f>
+        <v/>
+      </c>
+      <c r="H9" s="59"/>
+      <c r="I9" s="59">
+        <f>'Class Roster'!K13</f>
+        <v>126</v>
+      </c>
     </row>
     <row r="10">
-      <c r="B10" s="55"/>
-      <c r="C10" s="67"/>
-      <c r="D10" s="55"/>
-      <c r="E10" s="55"/>
-      <c r="F10" s="55"/>
-      <c r="G10" s="55"/>
-      <c r="H10" s="55"/>
-      <c r="I10" s="55"/>
+      <c r="B10" s="59" t="str">
+        <f t="array" ref="B10:C10">'Class Roster'!C14:D14</f>
+        <v/>
+      </c>
+      <c r="C10" s="63"/>
+      <c r="D10" s="59" t="str">
+        <f t="array" ref="D10:F10">'Class Roster'!G14:I14</f>
+        <v/>
+      </c>
+      <c r="E10" s="59"/>
+      <c r="F10" s="59"/>
+      <c r="G10" s="59" t="str">
+        <f t="array" ref="G10:H10">'Student List'!I11:J11</f>
+        <v/>
+      </c>
+      <c r="H10" s="59"/>
+      <c r="I10" s="59">
+        <f>'Class Roster'!K14</f>
+        <v>126</v>
+      </c>
     </row>
     <row r="11">
-      <c r="B11" s="55"/>
-      <c r="C11" s="55"/>
-      <c r="D11" s="55"/>
-      <c r="E11" s="55"/>
-      <c r="F11" s="55"/>
-      <c r="G11" s="55"/>
-      <c r="H11" s="55"/>
-      <c r="I11" s="55"/>
+      <c r="B11" s="59" t="str">
+        <f t="array" ref="B11:C11">'Class Roster'!C15:D15</f>
+        <v/>
+      </c>
+      <c r="C11" s="59"/>
+      <c r="D11" s="59" t="str">
+        <f t="array" ref="D11:F11">'Class Roster'!G15:I15</f>
+        <v/>
+      </c>
+      <c r="E11" s="59"/>
+      <c r="F11" s="59"/>
+      <c r="G11" s="59" t="str">
+        <f t="array" ref="G11:H11">'Student List'!I12:J12</f>
+        <v/>
+      </c>
+      <c r="H11" s="59"/>
+      <c r="I11" s="59">
+        <f>'Class Roster'!K15</f>
+        <v>126</v>
+      </c>
     </row>
     <row r="12">
-      <c r="B12" s="55"/>
-      <c r="C12" s="55"/>
-      <c r="D12" s="55"/>
-      <c r="E12" s="55"/>
-      <c r="F12" s="55"/>
-      <c r="G12" s="55"/>
-      <c r="H12" s="55"/>
-      <c r="I12" s="55"/>
+      <c r="B12" s="59" t="str">
+        <f t="array" ref="B12:C12">'Class Roster'!C16:D16</f>
+        <v/>
+      </c>
+      <c r="C12" s="59"/>
+      <c r="D12" s="59" t="str">
+        <f t="array" ref="D12:F12">'Class Roster'!G16:I16</f>
+        <v/>
+      </c>
+      <c r="E12" s="59"/>
+      <c r="F12" s="59"/>
+      <c r="G12" s="59" t="str">
+        <f t="array" ref="G12:H12">'Student List'!I13:J13</f>
+        <v/>
+      </c>
+      <c r="H12" s="59"/>
+      <c r="I12" s="59">
+        <f>'Class Roster'!K16</f>
+        <v>126</v>
+      </c>
     </row>
     <row r="13">
-      <c r="B13" s="55"/>
-      <c r="C13" s="55"/>
-      <c r="D13" s="55"/>
-      <c r="E13" s="55"/>
-      <c r="F13" s="55"/>
-      <c r="G13" s="55"/>
-      <c r="H13" s="55"/>
-      <c r="I13" s="55"/>
+      <c r="B13" s="59" t="str">
+        <f t="array" ref="B13:C13">'Class Roster'!C17:D17</f>
+        <v/>
+      </c>
+      <c r="C13" s="59"/>
+      <c r="D13" s="59" t="str">
+        <f t="array" ref="D13:F13">'Class Roster'!G17:I17</f>
+        <v/>
+      </c>
+      <c r="E13" s="59"/>
+      <c r="F13" s="59"/>
+      <c r="G13" s="59" t="str">
+        <f t="array" ref="G13:H13">'Student List'!I14:J14</f>
+        <v/>
+      </c>
+      <c r="H13" s="59"/>
+      <c r="I13" s="59">
+        <f>'Class Roster'!K17</f>
+        <v>126</v>
+      </c>
     </row>
     <row r="14">
-      <c r="B14" s="55"/>
-      <c r="C14" s="55"/>
-      <c r="D14" s="55"/>
-      <c r="E14" s="55"/>
-      <c r="F14" s="55"/>
-      <c r="G14" s="55"/>
-      <c r="H14" s="55"/>
-      <c r="I14" s="55"/>
+      <c r="B14" s="59" t="str">
+        <f t="array" ref="B14:C14">'Class Roster'!C18:D18</f>
+        <v/>
+      </c>
+      <c r="C14" s="59"/>
+      <c r="D14" s="59" t="str">
+        <f t="array" ref="D14:F14">'Class Roster'!G18:I18</f>
+        <v/>
+      </c>
+      <c r="E14" s="59"/>
+      <c r="F14" s="59"/>
+      <c r="G14" s="59" t="str">
+        <f t="array" ref="G14:H14">'Student List'!I15:J15</f>
+        <v/>
+      </c>
+      <c r="H14" s="59"/>
+      <c r="I14" s="59">
+        <f>'Class Roster'!K18</f>
+        <v>126</v>
+      </c>
     </row>
     <row r="15">
-      <c r="B15" s="55"/>
-      <c r="C15" s="55"/>
-      <c r="D15" s="55"/>
-      <c r="E15" s="55"/>
-      <c r="F15" s="55"/>
-      <c r="G15" s="55"/>
-      <c r="H15" s="55"/>
-      <c r="I15" s="55"/>
+      <c r="B15" s="59" t="str">
+        <f t="array" ref="B15:C15">'Class Roster'!C19:D19</f>
+        <v/>
+      </c>
+      <c r="C15" s="59"/>
+      <c r="D15" s="59" t="str">
+        <f t="array" ref="D15:F15">'Class Roster'!G19:I19</f>
+        <v/>
+      </c>
+      <c r="E15" s="59"/>
+      <c r="F15" s="59"/>
+      <c r="G15" s="59" t="str">
+        <f t="array" ref="G15:H15">'Student List'!I16:J16</f>
+        <v/>
+      </c>
+      <c r="H15" s="59"/>
+      <c r="I15" s="59">
+        <f>'Class Roster'!K19</f>
+        <v>126</v>
+      </c>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>
@@ -19822,484 +20170,520 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="68"/>
-      <c r="B1" s="68"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="70"/>
-      <c r="E1" s="70"/>
-      <c r="F1" s="70"/>
-      <c r="G1" s="70"/>
-      <c r="H1" s="70"/>
-      <c r="I1" s="70"/>
-      <c r="J1" s="70"/>
-      <c r="K1" s="71"/>
-      <c r="L1" s="68"/>
-      <c r="M1" s="68"/>
-      <c r="N1" s="68"/>
-      <c r="O1" s="68"/>
+      <c r="A1" s="64"/>
+      <c r="B1" s="64"/>
+      <c r="C1" s="65"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="66"/>
+      <c r="J1" s="66"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="64"/>
+      <c r="M1" s="64"/>
+      <c r="N1" s="64"/>
+      <c r="O1" s="64"/>
     </row>
     <row r="2">
-      <c r="A2" s="72" t="s">
+      <c r="A2" s="68" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="73"/>
-      <c r="C2" s="68"/>
-      <c r="D2" s="68"/>
-      <c r="E2" s="68"/>
-      <c r="F2" s="68"/>
-      <c r="G2" s="68"/>
-      <c r="H2" s="68"/>
-      <c r="I2" s="68"/>
-      <c r="J2" s="74"/>
-      <c r="K2" s="68"/>
-      <c r="L2" s="68"/>
-      <c r="M2" s="68"/>
-      <c r="N2" s="68"/>
-      <c r="O2" s="68"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="64"/>
+      <c r="D2" s="64"/>
+      <c r="E2" s="64"/>
+      <c r="F2" s="64"/>
+      <c r="G2" s="64"/>
+      <c r="H2" s="64"/>
+      <c r="I2" s="64"/>
+      <c r="J2" s="70"/>
+      <c r="K2" s="64"/>
+      <c r="L2" s="64"/>
+      <c r="M2" s="64"/>
+      <c r="N2" s="64"/>
+      <c r="O2" s="64"/>
     </row>
     <row r="3">
-      <c r="A3" s="75"/>
-      <c r="B3" s="76"/>
-      <c r="C3" s="77" t="s">
+      <c r="A3" s="71"/>
+      <c r="B3" s="72"/>
+      <c r="C3" s="73" t="s">
         <v>30</v>
       </c>
-      <c r="D3" s="77" t="s">
+      <c r="D3" s="73" t="s">
         <v>31</v>
       </c>
-      <c r="E3" s="77" t="s">
+      <c r="E3" s="73" t="s">
         <v>30</v>
       </c>
-      <c r="F3" s="77" t="s">
+      <c r="F3" s="73" t="s">
         <v>31</v>
       </c>
-      <c r="G3" s="77" t="s">
+      <c r="G3" s="73" t="s">
         <v>30</v>
       </c>
-      <c r="H3" s="77" t="s">
+      <c r="H3" s="73" t="s">
         <v>31</v>
       </c>
-      <c r="I3" s="77" t="s">
+      <c r="I3" s="73" t="s">
         <v>30</v>
       </c>
-      <c r="J3" s="77" t="s">
+      <c r="J3" s="73" t="s">
         <v>31</v>
       </c>
-      <c r="K3" s="78" t="s">
+      <c r="K3" s="74" t="s">
         <v>32</v>
       </c>
-      <c r="L3" s="79" t="s">
+      <c r="L3" s="75" t="s">
         <v>33</v>
       </c>
-      <c r="M3" s="80" t="s">
+      <c r="M3" s="76" t="s">
         <v>34</v>
       </c>
-      <c r="N3" s="81" t="s">
+      <c r="N3" s="77" t="s">
         <v>35</v>
       </c>
-      <c r="O3" s="82" t="s">
+      <c r="O3" s="78" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="83" t="s">
+      <c r="A4" s="79" t="s">
         <v>37</v>
       </c>
-      <c r="B4" s="83" t="s">
+      <c r="B4" s="79" t="s">
         <v>38</v>
       </c>
-      <c r="C4" s="77" t="s">
+      <c r="C4" s="73" t="s">
         <v>39</v>
       </c>
-      <c r="D4" s="77" t="s">
+      <c r="D4" s="73" t="s">
         <v>40</v>
       </c>
-      <c r="E4" s="77" t="s">
+      <c r="E4" s="73" t="s">
         <v>41</v>
       </c>
-      <c r="F4" s="77" t="s">
+      <c r="F4" s="73" t="s">
         <v>42</v>
       </c>
-      <c r="G4" s="77" t="s">
+      <c r="G4" s="73" t="s">
         <v>43</v>
       </c>
-      <c r="H4" s="77" t="s">
+      <c r="H4" s="73" t="s">
         <v>44</v>
       </c>
-      <c r="I4" s="77" t="s">
+      <c r="I4" s="73" t="s">
         <v>45</v>
       </c>
-      <c r="J4" s="77" t="s">
+      <c r="J4" s="73" t="s">
         <v>46</v>
       </c>
-      <c r="K4" s="84"/>
-      <c r="L4" s="84"/>
-      <c r="M4" s="84"/>
-      <c r="N4" s="84"/>
-      <c r="O4" s="84"/>
+      <c r="K4" s="80"/>
+      <c r="L4" s="80"/>
+      <c r="M4" s="80"/>
+      <c r="N4" s="80"/>
+      <c r="O4" s="80"/>
     </row>
     <row r="5">
-      <c r="A5" s="85"/>
-      <c r="B5" s="86"/>
+      <c r="A5" s="81" t="str">
+        <f t="array" ref="A5:B5">'Class Roster'!C8:D8</f>
+        <v/>
+      </c>
+      <c r="B5" s="82"/>
       <c r="C5" s="32"/>
       <c r="D5" s="32"/>
-      <c r="E5" s="41"/>
-      <c r="F5" s="41"/>
-      <c r="G5" s="41"/>
-      <c r="H5" s="41"/>
-      <c r="I5" s="41"/>
-      <c r="J5" s="41"/>
-      <c r="K5" s="87">
+      <c r="E5" s="44"/>
+      <c r="F5" s="44"/>
+      <c r="G5" s="44"/>
+      <c r="H5" s="44"/>
+      <c r="I5" s="44"/>
+      <c r="J5" s="44"/>
+      <c r="K5" s="83">
         <f t="shared" ref="K5:K9" si="1">COUNTA(C5:J5)-COUNTIF(C5:G5,"X")</f>
         <v>0</v>
       </c>
-      <c r="L5" s="88">
+      <c r="L5" s="84">
         <f t="shared" ref="L5:L16" si="2">COUNTIF(C5:J5,"X")</f>
         <v>0</v>
       </c>
-      <c r="M5" s="89" t="str">
+      <c r="M5" s="85" t="str">
         <f t="shared" ref="M5:M16" si="3">K5/COUNTA(C5:J5)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="N5" s="90" t="str">
+      <c r="N5" s="86" t="str">
         <f t="shared" ref="N5:N16" si="4">L5/COUNTA(C5:J5)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="O5" s="41"/>
+      <c r="O5" s="44"/>
     </row>
     <row r="6">
-      <c r="A6" s="85"/>
-      <c r="B6" s="85"/>
+      <c r="A6" s="81" t="str">
+        <f t="array" ref="A6:B6">'Class Roster'!C9:D9</f>
+        <v/>
+      </c>
+      <c r="B6" s="81"/>
       <c r="C6" s="32"/>
       <c r="D6" s="32"/>
-      <c r="E6" s="41"/>
-      <c r="F6" s="41"/>
-      <c r="G6" s="41"/>
-      <c r="H6" s="41"/>
-      <c r="I6" s="41"/>
-      <c r="J6" s="41"/>
-      <c r="K6" s="87">
+      <c r="E6" s="44"/>
+      <c r="F6" s="44"/>
+      <c r="G6" s="44"/>
+      <c r="H6" s="44"/>
+      <c r="I6" s="44"/>
+      <c r="J6" s="44"/>
+      <c r="K6" s="83">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="L6" s="88">
+      <c r="L6" s="84">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M6" s="89" t="str">
+      <c r="M6" s="85" t="str">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="N6" s="90" t="str">
+      <c r="N6" s="86" t="str">
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="O6" s="41"/>
+      <c r="O6" s="44"/>
     </row>
     <row r="7">
-      <c r="A7" s="85"/>
-      <c r="B7" s="85"/>
+      <c r="A7" s="81" t="str">
+        <f t="array" ref="A7:B7">'Class Roster'!C10:D10</f>
+        <v/>
+      </c>
+      <c r="B7" s="81"/>
       <c r="C7" s="32"/>
       <c r="D7" s="32"/>
-      <c r="E7" s="41"/>
-      <c r="F7" s="41"/>
-      <c r="G7" s="41"/>
-      <c r="H7" s="41"/>
-      <c r="I7" s="41"/>
-      <c r="J7" s="41"/>
-      <c r="K7" s="87">
+      <c r="E7" s="44"/>
+      <c r="F7" s="44"/>
+      <c r="G7" s="44"/>
+      <c r="H7" s="44"/>
+      <c r="I7" s="44"/>
+      <c r="J7" s="44"/>
+      <c r="K7" s="83">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="L7" s="88">
+      <c r="L7" s="84">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M7" s="89" t="str">
+      <c r="M7" s="85" t="str">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="N7" s="90" t="str">
+      <c r="N7" s="86" t="str">
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="O7" s="41"/>
+      <c r="O7" s="44"/>
     </row>
     <row r="8">
-      <c r="A8" s="85"/>
-      <c r="B8" s="85"/>
+      <c r="A8" s="81" t="str">
+        <f t="array" ref="A8:B8">'Class Roster'!C11:D11</f>
+        <v/>
+      </c>
+      <c r="B8" s="81"/>
       <c r="C8" s="32"/>
       <c r="D8" s="32"/>
-      <c r="E8" s="41"/>
-      <c r="F8" s="41"/>
-      <c r="G8" s="41"/>
-      <c r="H8" s="41"/>
-      <c r="I8" s="41"/>
-      <c r="J8" s="41"/>
-      <c r="K8" s="87">
+      <c r="E8" s="44"/>
+      <c r="F8" s="44"/>
+      <c r="G8" s="44"/>
+      <c r="H8" s="44"/>
+      <c r="I8" s="44"/>
+      <c r="J8" s="44"/>
+      <c r="K8" s="83">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="L8" s="88">
+      <c r="L8" s="84">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M8" s="89" t="str">
+      <c r="M8" s="85" t="str">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="N8" s="90" t="str">
+      <c r="N8" s="86" t="str">
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="O8" s="41"/>
+      <c r="O8" s="44"/>
     </row>
     <row r="9">
-      <c r="A9" s="85"/>
-      <c r="B9" s="85"/>
+      <c r="A9" s="81" t="str">
+        <f t="array" ref="A9:B9">'Class Roster'!C12:D12</f>
+        <v/>
+      </c>
+      <c r="B9" s="81"/>
       <c r="C9" s="32"/>
       <c r="D9" s="32"/>
-      <c r="E9" s="41"/>
-      <c r="F9" s="41"/>
-      <c r="G9" s="41"/>
-      <c r="H9" s="41"/>
-      <c r="I9" s="41"/>
-      <c r="J9" s="41"/>
-      <c r="K9" s="87">
+      <c r="E9" s="44"/>
+      <c r="F9" s="44"/>
+      <c r="G9" s="44"/>
+      <c r="H9" s="44"/>
+      <c r="I9" s="44"/>
+      <c r="J9" s="44"/>
+      <c r="K9" s="83">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="L9" s="88">
+      <c r="L9" s="84">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M9" s="89" t="str">
+      <c r="M9" s="85" t="str">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="N9" s="90" t="str">
+      <c r="N9" s="86" t="str">
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="O9" s="41"/>
+      <c r="O9" s="44"/>
     </row>
     <row r="10">
-      <c r="A10" s="85"/>
-      <c r="B10" s="85"/>
+      <c r="A10" s="81" t="str">
+        <f t="array" ref="A10:B10">'Class Roster'!C13:D13</f>
+        <v/>
+      </c>
+      <c r="B10" s="81"/>
       <c r="C10" s="32"/>
       <c r="D10" s="32"/>
-      <c r="E10" s="41"/>
-      <c r="F10" s="41"/>
-      <c r="G10" s="41"/>
-      <c r="H10" s="41"/>
-      <c r="I10" s="41"/>
-      <c r="J10" s="41"/>
-      <c r="K10" s="87">
+      <c r="E10" s="44"/>
+      <c r="F10" s="44"/>
+      <c r="G10" s="44"/>
+      <c r="H10" s="44"/>
+      <c r="I10" s="44"/>
+      <c r="J10" s="44"/>
+      <c r="K10" s="83">
         <f>COUNTIF(C10:J10, "O")</f>
         <v>0</v>
       </c>
-      <c r="L10" s="88">
+      <c r="L10" s="84">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M10" s="89" t="str">
+      <c r="M10" s="85" t="str">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="N10" s="90" t="str">
+      <c r="N10" s="86" t="str">
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="O10" s="41"/>
+      <c r="O10" s="44"/>
     </row>
     <row r="11">
-      <c r="A11" s="85"/>
-      <c r="B11" s="86"/>
+      <c r="A11" s="81" t="str">
+        <f t="array" ref="A11:B11">'Class Roster'!C14:D14</f>
+        <v/>
+      </c>
+      <c r="B11" s="82"/>
       <c r="C11" s="32"/>
       <c r="D11" s="32"/>
-      <c r="E11" s="41"/>
-      <c r="F11" s="41"/>
-      <c r="G11" s="41"/>
-      <c r="H11" s="41"/>
-      <c r="I11" s="41"/>
-      <c r="J11" s="41"/>
-      <c r="K11" s="87">
+      <c r="E11" s="44"/>
+      <c r="F11" s="44"/>
+      <c r="G11" s="44"/>
+      <c r="H11" s="44"/>
+      <c r="I11" s="44"/>
+      <c r="J11" s="44"/>
+      <c r="K11" s="83">
         <f t="shared" ref="K11:K16" si="5">COUNTA(C11:J11)-COUNTIF(C11:G11,"X")</f>
         <v>0</v>
       </c>
-      <c r="L11" s="88">
+      <c r="L11" s="84">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M11" s="89" t="str">
+      <c r="M11" s="85" t="str">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="N11" s="90" t="str">
+      <c r="N11" s="86" t="str">
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="O11" s="41"/>
+      <c r="O11" s="44"/>
     </row>
     <row r="12">
-      <c r="A12" s="85"/>
-      <c r="B12" s="85"/>
+      <c r="A12" s="81" t="str">
+        <f t="array" ref="A12:B12">'Class Roster'!C15:D15</f>
+        <v/>
+      </c>
+      <c r="B12" s="81"/>
       <c r="C12" s="32"/>
       <c r="D12" s="32"/>
-      <c r="E12" s="41"/>
-      <c r="F12" s="41"/>
-      <c r="G12" s="41"/>
-      <c r="H12" s="41"/>
-      <c r="I12" s="41"/>
-      <c r="J12" s="41"/>
-      <c r="K12" s="87">
+      <c r="E12" s="44"/>
+      <c r="F12" s="44"/>
+      <c r="G12" s="44"/>
+      <c r="H12" s="44"/>
+      <c r="I12" s="44"/>
+      <c r="J12" s="44"/>
+      <c r="K12" s="83">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="L12" s="88">
+      <c r="L12" s="84">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M12" s="89" t="str">
+      <c r="M12" s="85" t="str">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="N12" s="90" t="str">
+      <c r="N12" s="86" t="str">
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="O12" s="41"/>
+      <c r="O12" s="44"/>
     </row>
     <row r="13">
-      <c r="A13" s="85"/>
-      <c r="B13" s="85"/>
-      <c r="C13" s="41"/>
-      <c r="D13" s="41"/>
-      <c r="E13" s="41"/>
-      <c r="F13" s="41"/>
-      <c r="G13" s="41"/>
-      <c r="H13" s="41"/>
-      <c r="I13" s="41"/>
-      <c r="J13" s="41"/>
-      <c r="K13" s="87">
+      <c r="A13" s="81" t="str">
+        <f t="array" ref="A13:B13">'Class Roster'!C16:D16</f>
+        <v/>
+      </c>
+      <c r="B13" s="81"/>
+      <c r="C13" s="44"/>
+      <c r="D13" s="44"/>
+      <c r="E13" s="44"/>
+      <c r="F13" s="44"/>
+      <c r="G13" s="44"/>
+      <c r="H13" s="44"/>
+      <c r="I13" s="44"/>
+      <c r="J13" s="44"/>
+      <c r="K13" s="83">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="L13" s="88">
+      <c r="L13" s="84">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M13" s="89" t="str">
+      <c r="M13" s="85" t="str">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="N13" s="90" t="str">
+      <c r="N13" s="86" t="str">
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="O13" s="41"/>
+      <c r="O13" s="44"/>
     </row>
     <row r="14">
-      <c r="A14" s="85"/>
-      <c r="B14" s="85"/>
-      <c r="C14" s="41"/>
-      <c r="D14" s="41"/>
-      <c r="E14" s="41"/>
-      <c r="F14" s="41"/>
-      <c r="G14" s="41"/>
-      <c r="H14" s="41"/>
-      <c r="I14" s="41"/>
-      <c r="J14" s="41"/>
-      <c r="K14" s="87">
+      <c r="A14" s="81" t="str">
+        <f t="array" ref="A14:B14">'Class Roster'!C17:D17</f>
+        <v/>
+      </c>
+      <c r="B14" s="81"/>
+      <c r="C14" s="44"/>
+      <c r="D14" s="44"/>
+      <c r="E14" s="44"/>
+      <c r="F14" s="44"/>
+      <c r="G14" s="44"/>
+      <c r="H14" s="44"/>
+      <c r="I14" s="44"/>
+      <c r="J14" s="44"/>
+      <c r="K14" s="83">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="L14" s="88">
+      <c r="L14" s="84">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M14" s="89" t="str">
+      <c r="M14" s="85" t="str">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="N14" s="90" t="str">
+      <c r="N14" s="86" t="str">
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="O14" s="41"/>
+      <c r="O14" s="44"/>
     </row>
     <row r="15">
-      <c r="A15" s="85"/>
-      <c r="B15" s="85"/>
-      <c r="C15" s="41"/>
-      <c r="D15" s="41"/>
-      <c r="E15" s="41"/>
-      <c r="F15" s="41"/>
-      <c r="G15" s="41"/>
-      <c r="H15" s="41"/>
-      <c r="I15" s="41"/>
-      <c r="J15" s="41"/>
-      <c r="K15" s="87">
+      <c r="A15" s="81" t="str">
+        <f t="array" ref="A15:B15">'Class Roster'!C18:D18</f>
+        <v/>
+      </c>
+      <c r="B15" s="81"/>
+      <c r="C15" s="44"/>
+      <c r="D15" s="44"/>
+      <c r="E15" s="44"/>
+      <c r="F15" s="44"/>
+      <c r="G15" s="44"/>
+      <c r="H15" s="44"/>
+      <c r="I15" s="44"/>
+      <c r="J15" s="44"/>
+      <c r="K15" s="83">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="L15" s="88">
+      <c r="L15" s="84">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M15" s="89" t="str">
+      <c r="M15" s="85" t="str">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="N15" s="90" t="str">
+      <c r="N15" s="86" t="str">
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="O15" s="41"/>
+      <c r="O15" s="44"/>
     </row>
     <row r="16" ht="15.75" customHeight="1">
-      <c r="A16" s="85"/>
-      <c r="B16" s="85"/>
-      <c r="C16" s="41"/>
-      <c r="D16" s="41"/>
-      <c r="E16" s="41"/>
-      <c r="F16" s="41"/>
-      <c r="G16" s="41"/>
-      <c r="H16" s="41"/>
-      <c r="I16" s="41"/>
-      <c r="J16" s="41"/>
-      <c r="K16" s="87">
+      <c r="A16" s="81" t="str">
+        <f t="array" ref="A16:B16">'Class Roster'!C19:D19</f>
+        <v/>
+      </c>
+      <c r="B16" s="81"/>
+      <c r="C16" s="44"/>
+      <c r="D16" s="44"/>
+      <c r="E16" s="44"/>
+      <c r="F16" s="44"/>
+      <c r="G16" s="44"/>
+      <c r="H16" s="44"/>
+      <c r="I16" s="44"/>
+      <c r="J16" s="44"/>
+      <c r="K16" s="83">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="L16" s="88">
+      <c r="L16" s="84">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="M16" s="89" t="str">
+      <c r="M16" s="85" t="str">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="N16" s="90" t="str">
+      <c r="N16" s="86" t="str">
         <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="O16" s="41"/>
+      <c r="O16" s="44"/>
     </row>
     <row r="18">
-      <c r="A18" s="91" t="s">
+      <c r="A18" s="87" t="s">
         <v>47</v>
       </c>
-      <c r="B18" s="92" t="s">
+      <c r="B18" s="88" t="s">
         <v>48</v>
       </c>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
     </row>
     <row r="19">
-      <c r="A19" s="93" t="s">
+      <c r="A19" s="89" t="s">
         <v>49</v>
       </c>
-      <c r="B19" s="92" t="s">
+      <c r="B19" s="88" t="s">
         <v>50</v>
       </c>
       <c r="C19" s="1"/>
@@ -20308,8 +20692,8 @@
       <c r="F19" s="1"/>
     </row>
     <row r="20">
-      <c r="A20" s="94"/>
-      <c r="B20" s="92" t="s">
+      <c r="A20" s="90"/>
+      <c r="B20" s="88" t="s">
         <v>51</v>
       </c>
       <c r="C20" s="1"/>
@@ -20318,8 +20702,8 @@
       <c r="F20" s="1"/>
     </row>
     <row r="21">
-      <c r="A21" s="95"/>
-      <c r="B21" s="92" t="s">
+      <c r="A21" s="91"/>
+      <c r="B21" s="88" t="s">
         <v>52</v>
       </c>
       <c r="C21" s="1"/>

</xml_diff>